<commit_message>
Add reasoning tokens and GitHub commit attribution by agent type
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic_ai_revenue_token_usage_2026.xlsx
+++ b/agentic_ai_revenue_token_usage_2026.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Offerings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sector Aggregates" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Token Usage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offerings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sector Aggregates" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Usage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reasoning Tokens" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub Commits" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Offerings'!$A$1:$P$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Token Usage'!$A$1:$F$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reasoning Tokens'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'GitHub Commits'!$A$1:$L$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -575,125 +579,174 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Reasoning Tokens - reasoning-token consumption by agent type/workload (router-wide shares, per-task splits, stage-level intensity).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GitHub Commits - commit attribution per coding agent (WoC census V2510/V2604 windows, all-time attributed units, dev adoption).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Sources - numbered source list; the 'Sources' column in other sheets references these numbers.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>DEFINITIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ARR - annual recurring revenue as disclosed or estimated; in AI, often used interchangeably with annualized run-rate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Annualized run-rate - most recent period revenue x 12 (or x4); volatile for fast-growing companies.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tracked ARR - third-party estimate (e.g., TickerTrends) anchored to a company disclosure and extrapolated from usage signals.</t>
+          <t xml:space="preserve">  ARR - annual recurring revenue as disclosed or estimated; in AI, often used interchangeably with annualized run-rate.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Annualized run-rate - most recent period revenue x 12 (or x4); volatile for fast-growing companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tracked ARR - third-party estimate (e.g., TickerTrends) anchored to a company disclosure and extrapolated from usage signals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  ACV - annual contract value (ServiceNow reports its AI portfolio this way).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>KEY CAVEATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Double counting: model-provider totals (OpenAI, Anthropic, Google) overlap with application rows (Codex, Claude Code) and with</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     startups that resell frontier models (Cursor, Replit, Lovable pay API costs to providers). Memo rows are excluded from aggregates.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. Estimate quality varies: figures range from company-disclosed (Agentforce, Glean) to analyst-tracked (Claude Code, Codex) to</t>
+          <t xml:space="preserve">  1. Double counting: model-provider totals (OpenAI, Anthropic, Google) overlap with application rows (Codex, Claude Code) and with</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     analyst-inferred (Rogo). See the Confidence column.</t>
+          <t xml:space="preserve">     startups that resell frontier models (Cursor, Replit, Lovable pay API costs to providers). Memo rows are excluded from aggregates.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. Microsoft 365 Copilot revenue is not disclosed; 30M+ seats at $30/user/mo list implies up to ~$10.8B annualized, but actual</t>
+          <t xml:space="preserve">  2. Estimate quality varies: figures range from company-disclosed (Agentforce, Glean) to analyst-tracked (Claude Code, Codex) to</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     discounted revenue is unknown, so it is excluded from sector aggregates (a large downward bias on the Enterprise platform sector).</t>
+          <t xml:space="preserve">     analyst-inferred (Rogo). See the Confidence column.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. Token metrics are heterogeneous: platform-wide (Google), API-only (OpenAI), router-visible (OpenRouter/Vercel see only traffic</t>
+          <t xml:space="preserve">  3. Microsoft 365 Copilot revenue is not disclosed; 30M+ seats at $30/user/mo list implies up to ~$10.8B annualized, but actual</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">     routed through them - a small single-digit % of global volume). Do not sum across rows.</t>
+          <t xml:space="preserve">     discounted revenue is unknown, so it is excluded from sector aggregates (a large downward bias on the Enterprise platform sector).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Some figures are stale (Abridge/Ambience May 2025; Manus Aug 2025); dates are given per row.</t>
+          <t xml:space="preserve">  4. Token metrics are heterogeneous: platform-wide (Google), API-only (OpenAI), router-visible (OpenRouter/Vercel see only traffic</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">     routed through them - a small single-digit % of global volume). Do not sum across rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. Some figures are stale (Abridge/Ambience May 2025; Manus Aug 2025); dates are given per row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  6. Run-rates in this market can double in a quarter; treat point-in-time numbers accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7. GitHub commit attribution systematically undercounts 'silent' agents: Cursor and IDE Copilot do not sign commits, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Codex surfaces via pull requests, not commits (its PR marker stopped appearing Nov 2025). PR and commit censuses capture</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     nearly disjoint agent populations - compare agents only within the same detection channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  8. 'Reasoning tokens' has two meanings: share of tokens served by reasoning-optimized models (OpenRouter, &gt;50%) vs reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     tokens inside completions (~21.6% of agentic SWE task tokens). The Reasoning Tokens sheet labels each metric explicitly.</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3834,1227 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Agent type / workload</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>As-of</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Context / notes</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Sources (#)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>All agent types (router-wide)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Share of tokens routed through reasoning-optimized models</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>&gt;50% of all OpenRouter tokens (vs ~0% in early Q1 2025)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Late 2025</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Measures tokens served by reasoning models, not reasoning tokens within outputs; driven by agent-style workflows (GPT-5, Claude 4.5, Gemini 3 era)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>All agent types (router-wide)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Top reasoning models by token volume</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>xAI Grok Code Fast 1 #1, then Gemini 2.5 Pro, Gemini 2.5 Flash, Grok 4 Fast, gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Late 2025</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Code-oriented reasoning models lead the category; rapid model turnover</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>All agent types (router-wide)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Completion-token growth per request</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>~3x increase, mostly due to reasoning tokens</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning tokens are billed inside completion tokens; programming workloads drive prompt growth (routinely &gt;20K input tokens/request)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (multi-agent SWE)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning share of task tokens</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>21.6% reasoning / 53.9% input / 24.4% output</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Jan 2026 (study)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>ChatDev framework + GPT-5 across 30 real development tasks</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (multi-agent SWE)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning tokens per task</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>17,280-40,000 reasoning tokens per software task</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Jan 2026 (study)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>400K context window, 128K max output configuration</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (multi-agent SWE)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Token consumption by SDLC stage</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Code review 59.4% of all tokens; code completion 26.8%; initial coding 8.6%; design 2.4%</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Jan 2026 (study)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Cost sits in automated refinement/verification, not initial generation</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (multi-agent SWE)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning intensity by stage</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Initial coding ~35% reasoning; code review ~23%; documentation ~6%</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Jan 2026 (study)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Generative stages are reasoning-heavy; analysis stages are input-heavy (documentation 80.2% input)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>44, 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (single-agent loops)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Token mix by operation</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Reading/navigating code 76.1%; executing/testing 12.1%; editing 11.8%</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>SWE-Pruner measurements on real agent workloads; agents mostly re-read the codebase</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (single-agent loops)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Input-token dominance</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Input &gt;90-99% of trajectory volume; input:output ratio &gt;150:1</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Stateless loops re-send accumulated context every roundtrip; 99% of Claude 4 Sonnet's ~100B tokens/day on OpenRouter (Sep 2025) were input</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents vs chat</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Total token multiplier</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>~1,000x tokens vs a single-turn chat request</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Third-party token-economics research</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>23, 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Multi-agent systems vs chatbot</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Token multiplier</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Up to 15x tokens vs a chatbot request</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic estimate; consistent with OpenRouter's ~15x agentic-vs-human per-request measurement</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>23, 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Coding agents (task outcomes)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Failed vs successful task consumption</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Unresolved tasks: 697.7K tokens / 12.95 tool calls avg; resolved: 258.7K / 7.2 (2.7x gap)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>2026 (study)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>No positive correlation between token spend and success; failing patches trap agents in edit-test-read loops. Latest scaffold versions average ~668K tokens/task</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Configuration reference</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Reasoning-effort budget mapping</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>'low' ~20% of max_tokens for thinking; 'high' ~80%</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>OpenRouter API reasoning.effort parameter; reasoning tokens billed as output</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="56" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Deployment type</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Attribution channel</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Commits (cum. thru Oct 2025, WoC V2510)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Commits (Dec 2025-Apr 2026, WoC V2604)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>All-time attributed units (commits+PRs, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Developer adoption (May-Jul 2026)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Sources (#)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Claude Code</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>CLI / in-editor (commits directly)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Co-authored-by trailer + bot account (30x undercount if bot-only)</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>850157</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>886122</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>+4%</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>17,295</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>12.5M</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>39% of devs worldwide (47% US), up from 18% Jan 2026; most-used tool for 31%</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>50% of all AI-attributed commits in V2604; ~4% of ALL public GitHub commits (SemiAnalysis, Feb 2026), projected 20%+ of daily commits by end-2026; near-absent from PR channel (1.4% of AIDev agentic PRs)</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>41, 42, 43, 4, 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Copilot (SWE agent)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft (GitHub)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>PR-based cloud agent + IDE</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Bot account / workflow; IDE Copilot is commit-silent (config-file detection only)</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>1127201</v>
+      </c>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>n/a (not in V2604 table)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>85,739</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>3.8M</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>21% of devs, down from 29% a year ago; 79% awareness</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Largest agent in V2510 (2x Dependabot's volume); IDE Copilot appears in 92,276 projects via config files but &lt;0.5% of commits - silent-agent undercount</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>41, 42, 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Replit Agent</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Replit</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Auto-commits generated code (no PRs)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Message-signature template</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>312705</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>314779</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>+1% (flat)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Dominates explicit commit attribution among app-builder agents due to auto-commit workflow</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>41, 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Google Jules</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Async cloud agent</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Bot account / workflow</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>209911</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>215804</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>+3%</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>16,924</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Reached ~210K commits within nine months of launch</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Aider</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Open source</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>CLI pair-programmer</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Author-name suffix '(aider)'</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>195029</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>196132</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>+1% (flat)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>355 authors</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Only 4 config files in the entire corpus - invisible without author-name scanning; skews to existing repos rather than greenfield</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Devin (+ Windsurf)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Cognition</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Autonomous cloud engineer (PR + commit channels)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Bot account (devin-ai-integration[bot]) + conventional commits</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>215998</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>98493</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>-54%</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>7,050</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>256.4K</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Uses both PR and commit channels (3,657 shared repos); V2604 window volume fell by half; 14.4% of AIDev agentic PRs</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>41, 42, 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>CodeRabbit</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>CodeRabbit</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Code-review agent</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Bot account</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>297</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>34940</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>+117x</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Fastest-growing commit-attributed agent between snapshots (review-agent category emerging)</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>OpenHands</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>All Hands AI</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Open-source autonomous agent</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Bot account</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>20863</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>25676</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>+23%</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>1,022</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Predominantly used in born-with-AI greenfield repositories</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PR-based cloud agent</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>PR body marker (stopped appearing Nov 2025); no commit attribution</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>843</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>731</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>-13%</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>5.1M</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>16% of devs, up from 3% Jan 2026; awareness 27% -&gt; 65%</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Mirror image of Claude Code: largest agent by PULL REQUESTS (814,522 in AIDev; 64.9% of agentic PRs) yet near-absent from commit data - commit census misses essentially all Codex adopters; all-time units undercounted since Nov 2025</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>41, 42, 43, 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Cursor (agent mode)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Anysphere</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>IDE agent</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>None by default (commit-silent); .cursorrules config detection</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>28,909 (config)</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Zero attributed commits; 32,941 PRs in AIDev (4.6% of agentic PRs); a major example of attribution undercounting silent agents</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>41, 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Dependabot (control)</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Non-LLM dependency bot (baseline)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Bot account</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>475379</v>
+      </c>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>44,731</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="7" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Non-AI control baseline active since 2017; Copilot SWE agent alone now exceeds 2x its cumulative volume</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>(Ecosystem) All AI agents</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n">
+        <v>1772677</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>315,426 projects</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>27.1M (all agents)</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>1.77M commit-attributed AI commits in Dec 2025-Apr 2026; &gt;320K AI commits/month by mid-2025 (from 75K in Dec 2024); AI share of non-bot commits in adopting projects: 1.6% (Dec 2025) -&gt; 6.7% (Mar 2026)</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>41, 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>(Ecosystem) Agentic PR mix</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>AIDev-pop (Oct 2025) agentic PR share: Codex 64.9%, Copilot 14.8%, Devin 14.4%, Cursor 4.6%, Claude Code 1.4% - PR and commit censuses capture nearly disjoint agent populations</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4609,6 +5882,206 @@
       <c r="D41" s="16" t="inlineStr">
         <is>
           <t>https://www.beri.net/article/spacex-cursor-60b-acquisition-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2606.24429</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Detecting AI Coding Agents in Open Source: A Validated Multi-Method Census of 180M Repositories (WoC V2510/V2604)</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>https://www.alphaxiv.org/abs/2606.24429</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Amplifying.ai</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Coding Agents By Owner: all-time attributed commits + PRs per agent</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>https://amplifying.ai/coding-agents/public-companies</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>JetBrains Research</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>AI Coding Agents: Adoption Trends (Developer Ecosystem Survey, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>https://blog.jetbrains.com/research/2026/08/ai-coding-agent-adoption-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2601.14470</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Tokenomics: Quantifying Where Tokens Are Used in Agentic Software Engineering (ChatDev + GPT-5)</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arxiv.2601.14470</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>SaaSCity</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>59% of AI Agent Tokens Go to Code Review, Not Code Generation (Tokenomics coverage)</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>https://saascity.io/blog/tokenomics-quantifying-tokens-agentic-software-engineering-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>unerr</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Token optimization for AI coding agents (SWE-Pruner: reads 76.1% of agent tokens)</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>https://unerr.dev/blog/token-optimization-coding-agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Augment Code</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>AI Coding Cost Analysis: Where Token Spend Really Goes in an Agent Loop</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>https://www.augmentcode.com/guides/ai-coding-cost-analysis-agent-token-spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2601.17406</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Fingerprinting AI Coding Agents on GitHub (AIDev-pop PR mix by agent)</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arxiv.2601.17406</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2507.15003</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>The Rise of AI Teammates in SE 3.0 (agent attribution channels)</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/html/2507.15003v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>arXiv 2607.03691</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Scaffolding Evolution &amp; Coding Agent Quality (failed tasks consume 2.7x tokens)</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.48550/arxiv.2607.03691</t>
         </is>
       </c>
     </row>
@@ -4654,6 +6127,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>